<commit_message>
Implemented fixes to allow older case to run in latest Macro, updated readmes, dev to stable
</commit_message>
<xml_diff>
--- a/electricity_fiveZ_8736_1p_nziShadow_stable/viz_compare_info/0_NZIshadow_PIERinfo.xlsx
+++ b/electricity_fiveZ_8736_1p_nziShadow_stable/viz_compare_info/0_NZIshadow_PIERinfo.xlsx
@@ -5,18 +5,19 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\apascale\OneDrive - Princeton University\Documents\GitHub\NZx_caseDev_MacroEP\electricity_fiveZ_8736_1p_nziShadow_stable\viz_compare_info\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\apascale\OneDrive - Princeton University\Documents\GitHub\NZx_caseDev_MacroEP\electricity_fiveZ_8736_1p_nziShadow_dev\viz_compare_info\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D17A01DC-CEA0-4F9B-B950-23270873E845}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44E5FD2E-4BE6-4D78-9B70-396193CF5071}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{0C04E4D0-5751-44E6-BC3B-AD203EDB8BF9}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{0C04E4D0-5751-44E6-BC3B-AD203EDB8BF9}"/>
   </bookViews>
   <sheets>
     <sheet name="ECT_EfficiencyCostMaxAnnualUF" sheetId="1" r:id="rId1"/>
-    <sheet name="Carriers" sheetId="4" r:id="rId2"/>
-    <sheet name="Transmission" sheetId="3" r:id="rId3"/>
-    <sheet name="ECT_MaxAdd2024" sheetId="2" r:id="rId4"/>
+    <sheet name="Storage" sheetId="5" r:id="rId2"/>
+    <sheet name="Carriers" sheetId="4" r:id="rId3"/>
+    <sheet name="Transmission" sheetId="3" r:id="rId4"/>
+    <sheet name="ECT_MaxAdd2024" sheetId="2" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">ECT_EfficiencyCostMaxAnnualUF!#REF!</definedName>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="464" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="548" uniqueCount="156">
   <si>
     <t>EnergyConvTech</t>
   </si>
@@ -408,6 +409,105 @@
   </si>
   <si>
     <t>MW 2024</t>
+  </si>
+  <si>
+    <t>EnergyStorTech</t>
+  </si>
+  <si>
+    <t>StoredEC</t>
+  </si>
+  <si>
+    <t>DomOrImp</t>
+  </si>
+  <si>
+    <t>MaxChargeRate</t>
+  </si>
+  <si>
+    <t>MaxDischargeRate</t>
+  </si>
+  <si>
+    <t>StorPeriodicity</t>
+  </si>
+  <si>
+    <t>Comment</t>
+  </si>
+  <si>
+    <t>TWOHR_BATTERY</t>
+  </si>
+  <si>
+    <t>EC_DOM</t>
+  </si>
+  <si>
+    <t>DAILY</t>
+  </si>
+  <si>
+    <t>For now making all storages daily cycling - given computational constraints</t>
+  </si>
+  <si>
+    <t>FOURHR_BATTERY</t>
+  </si>
+  <si>
+    <t>SIXHR_BATTERY</t>
+  </si>
+  <si>
+    <t>PUMPED_STOR</t>
+  </si>
+  <si>
+    <t>Pumped storage discharges over 6 hours (Ensure latest info taken from EST Parameters workbook)</t>
+  </si>
+  <si>
+    <t>CapacityDerating</t>
+  </si>
+  <si>
+    <t>DepthOfDischarge</t>
+  </si>
+  <si>
+    <t>Efficiency</t>
+  </si>
+  <si>
+    <t>LegacyCapacity</t>
+  </si>
+  <si>
+    <t>BalLifetime</t>
+  </si>
+  <si>
+    <t>BalCycles</t>
+  </si>
+  <si>
+    <t>LifetimeYears</t>
+  </si>
+  <si>
+    <t>LifetimeCycles</t>
+  </si>
+  <si>
+    <t>EST_Lifetime.csv</t>
+  </si>
+  <si>
+    <t>EST_LegacyDetails.csv</t>
+  </si>
+  <si>
+    <t>EST_EfficiencyCost.csv</t>
+  </si>
+  <si>
+    <t>EST_DeratingDepthOfDischarge.csv</t>
+  </si>
+  <si>
+    <t>EnergyStorTechnologies.csv</t>
+  </si>
+  <si>
+    <t>File</t>
+  </si>
+  <si>
+    <t>PIER2.0</t>
+  </si>
+  <si>
+    <t>DischargeEfficiency</t>
+  </si>
+  <si>
+    <t>ChargeEfficiency</t>
+  </si>
+  <si>
+    <t>FixedCost (</t>
   </si>
 </sst>
 </file>
@@ -2750,6 +2850,472 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{167F2F9A-810A-4C8E-915E-BDC56D8F52B6}">
+  <dimension ref="A1:Q20"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17.28515625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="12" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="9.28515625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A1" s="10" t="s">
+        <v>90</v>
+      </c>
+      <c r="B1" t="s">
+        <v>152</v>
+      </c>
+      <c r="C1" t="s">
+        <v>152</v>
+      </c>
+      <c r="D1" t="s">
+        <v>152</v>
+      </c>
+      <c r="E1" t="s">
+        <v>152</v>
+      </c>
+      <c r="F1" t="s">
+        <v>152</v>
+      </c>
+      <c r="G1" t="s">
+        <v>152</v>
+      </c>
+      <c r="H1" t="s">
+        <v>152</v>
+      </c>
+      <c r="I1" t="s">
+        <v>152</v>
+      </c>
+      <c r="J1" t="s">
+        <v>152</v>
+      </c>
+      <c r="K1" t="s">
+        <v>152</v>
+      </c>
+      <c r="L1" t="s">
+        <v>152</v>
+      </c>
+      <c r="M1" t="s">
+        <v>152</v>
+      </c>
+      <c r="N1" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A2" s="10" t="s">
+        <v>151</v>
+      </c>
+      <c r="B2" t="s">
+        <v>150</v>
+      </c>
+      <c r="C2" t="s">
+        <v>150</v>
+      </c>
+      <c r="D2" t="s">
+        <v>150</v>
+      </c>
+      <c r="E2" t="s">
+        <v>150</v>
+      </c>
+      <c r="F2" t="s">
+        <v>150</v>
+      </c>
+      <c r="G2" t="s">
+        <v>150</v>
+      </c>
+      <c r="H2" t="s">
+        <v>149</v>
+      </c>
+      <c r="I2" t="s">
+        <v>149</v>
+      </c>
+      <c r="J2" t="s">
+        <v>149</v>
+      </c>
+      <c r="K2" t="s">
+        <v>148</v>
+      </c>
+      <c r="L2" t="s">
+        <v>148</v>
+      </c>
+      <c r="M2" t="s">
+        <v>146</v>
+      </c>
+      <c r="N2" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17" s="5" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>126</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>128</v>
+      </c>
+      <c r="G6" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="H6" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="I6" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="J6" s="5" t="s">
+        <v>139</v>
+      </c>
+      <c r="K6" s="5" t="s">
+        <v>155</v>
+      </c>
+      <c r="L6" s="5" t="s">
+        <v>140</v>
+      </c>
+      <c r="M6" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="N6" s="5" t="s">
+        <v>145</v>
+      </c>
+      <c r="P6" s="5" t="s">
+        <v>154</v>
+      </c>
+      <c r="Q6" s="5" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="7" spans="1:17" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>130</v>
+      </c>
+      <c r="B7" t="s">
+        <v>36</v>
+      </c>
+      <c r="C7" t="s">
+        <v>131</v>
+      </c>
+      <c r="D7">
+        <v>0.5</v>
+      </c>
+      <c r="E7">
+        <v>0.5</v>
+      </c>
+      <c r="F7" t="s">
+        <v>132</v>
+      </c>
+      <c r="G7" t="s">
+        <v>133</v>
+      </c>
+      <c r="H7">
+        <v>2024</v>
+      </c>
+      <c r="I7">
+        <v>0</v>
+      </c>
+      <c r="J7">
+        <v>0.9</v>
+      </c>
+      <c r="K7">
+        <f>2247.515108*1000</f>
+        <v>2247515.108</v>
+      </c>
+      <c r="L7">
+        <v>0.8</v>
+      </c>
+      <c r="M7" s="3">
+        <v>10</v>
+      </c>
+      <c r="N7">
+        <v>3873.4092000000001</v>
+      </c>
+    </row>
+    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>134</v>
+      </c>
+      <c r="B8" t="s">
+        <v>36</v>
+      </c>
+      <c r="C8" t="s">
+        <v>131</v>
+      </c>
+      <c r="D8">
+        <v>0.25</v>
+      </c>
+      <c r="E8">
+        <v>0.25</v>
+      </c>
+      <c r="F8" t="s">
+        <v>132</v>
+      </c>
+      <c r="H8">
+        <v>2024</v>
+      </c>
+      <c r="I8">
+        <v>0</v>
+      </c>
+      <c r="J8">
+        <v>0.9</v>
+      </c>
+      <c r="K8">
+        <v>1912.359346</v>
+      </c>
+      <c r="L8">
+        <v>0.8</v>
+      </c>
+      <c r="M8" s="3">
+        <v>10</v>
+      </c>
+      <c r="N8">
+        <v>3873.4092000000001</v>
+      </c>
+    </row>
+    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>135</v>
+      </c>
+      <c r="B9" t="s">
+        <v>36</v>
+      </c>
+      <c r="C9" t="s">
+        <v>131</v>
+      </c>
+      <c r="D9">
+        <v>0.16666700000000001</v>
+      </c>
+      <c r="E9">
+        <v>0.16666700000000001</v>
+      </c>
+      <c r="F9" t="s">
+        <v>132</v>
+      </c>
+      <c r="H9">
+        <v>2024</v>
+      </c>
+      <c r="I9">
+        <v>0</v>
+      </c>
+      <c r="J9">
+        <v>0.9</v>
+      </c>
+      <c r="K9">
+        <v>1800.6407589999999</v>
+      </c>
+      <c r="L9">
+        <v>0.8</v>
+      </c>
+      <c r="M9" s="3">
+        <v>10</v>
+      </c>
+      <c r="N9">
+        <v>3873.4092000000001</v>
+      </c>
+    </row>
+    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>136</v>
+      </c>
+      <c r="B10" t="s">
+        <v>36</v>
+      </c>
+      <c r="C10" t="s">
+        <v>131</v>
+      </c>
+      <c r="D10">
+        <v>0.16666666699999999</v>
+      </c>
+      <c r="E10">
+        <v>0.16666666699999999</v>
+      </c>
+      <c r="F10" t="s">
+        <v>132</v>
+      </c>
+      <c r="G10" t="s">
+        <v>137</v>
+      </c>
+      <c r="H10">
+        <v>2024</v>
+      </c>
+      <c r="I10">
+        <v>0</v>
+      </c>
+      <c r="J10">
+        <v>0.9</v>
+      </c>
+      <c r="K10">
+        <v>1900.130322</v>
+      </c>
+      <c r="L10">
+        <v>0.75</v>
+      </c>
+      <c r="M10" s="3">
+        <v>40</v>
+      </c>
+      <c r="N10">
+        <v>50000</v>
+      </c>
+      <c r="P10">
+        <f>SQRT(L10)</f>
+        <v>0.8660254037844386</v>
+      </c>
+      <c r="Q10">
+        <f>SQRT(L10)</f>
+        <v>0.8660254037844386</v>
+      </c>
+    </row>
+    <row r="14" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="15" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>123</v>
+      </c>
+      <c r="B15" t="s">
+        <v>1</v>
+      </c>
+      <c r="C15" t="s">
+        <v>2</v>
+      </c>
+      <c r="D15" t="s">
+        <v>141</v>
+      </c>
+      <c r="E15" t="s">
+        <v>142</v>
+      </c>
+      <c r="F15" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="16" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>136</v>
+      </c>
+      <c r="B16" t="s">
+        <v>7</v>
+      </c>
+      <c r="C16" t="s">
+        <v>11</v>
+      </c>
+      <c r="D16">
+        <v>5.4</v>
+      </c>
+      <c r="E16">
+        <v>20</v>
+      </c>
+      <c r="F16">
+        <v>50000</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>136</v>
+      </c>
+      <c r="B17" t="s">
+        <v>7</v>
+      </c>
+      <c r="C17" t="s">
+        <v>12</v>
+      </c>
+      <c r="D17">
+        <v>11.04</v>
+      </c>
+      <c r="E17">
+        <v>20</v>
+      </c>
+      <c r="F17">
+        <v>50000</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>136</v>
+      </c>
+      <c r="B18" t="s">
+        <v>7</v>
+      </c>
+      <c r="C18" t="s">
+        <v>10</v>
+      </c>
+      <c r="D18">
+        <v>0</v>
+      </c>
+      <c r="E18">
+        <v>20</v>
+      </c>
+      <c r="F18">
+        <v>50000</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>136</v>
+      </c>
+      <c r="B19" t="s">
+        <v>7</v>
+      </c>
+      <c r="C19" t="s">
+        <v>9</v>
+      </c>
+      <c r="D19">
+        <v>12.0336</v>
+      </c>
+      <c r="E19">
+        <v>20</v>
+      </c>
+      <c r="F19">
+        <v>50000</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>136</v>
+      </c>
+      <c r="B20" t="s">
+        <v>7</v>
+      </c>
+      <c r="C20" t="s">
+        <v>13</v>
+      </c>
+      <c r="D20">
+        <v>0</v>
+      </c>
+      <c r="E20">
+        <v>20</v>
+      </c>
+      <c r="F20">
+        <v>50000</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FD6847AC-1326-4512-A875-EA2269A8F204}">
   <dimension ref="A1:L22"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -3306,7 +3872,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E00B7979-01CA-4530-A3AC-4E09B913C2CA}">
   <dimension ref="A1:I26"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -4073,7 +4639,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{098E57D1-393A-4F40-8106-786EE712202A}">
   <dimension ref="A3:D75"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>

</xml_diff>